<commit_message>
Site updated: 2021-09-23 11:09:36
</commit_message>
<xml_diff>
--- a/games/life/data/achievement.xlsx
+++ b/games/life/data/achievement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\84694\Desktop\人生重来\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D59C89D-35FE-42A2-BD5F-BEA51D64AC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{192AAC15-664F-426D-8674-7964E8F2D586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="504">
   <si>
     <t>$id</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -1482,10 +1482,6 @@
   </si>
   <si>
     <t>信条</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>EVT?[11468,11469]</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
@@ -2024,10 +2020,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>(ATLT?[1023])&amp;(ATLT?[1048])&amp;(ATLT?[1064])&amp;(ATLT?[1114])&amp;(ATLT?[1135])</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>嫁衣</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -2053,6 +2045,38 @@
   </si>
   <si>
     <t>EVT?[40070]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EVT?[11468,11469,20390]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(ATLT?[1023])&amp;(ATLT?[1048])&amp;(ATLT?[1064])&amp;(ATLT?[1114])&amp;(ATLT?[1135])&amp;(ATLT?[1141])</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>有会员，所以急着投胎</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(TLT?[1122])&amp;(TLT?[1141])</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>薅羊毛专家</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>上当了</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TLT?[1136]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>太贪婪而被骗</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2440,7 +2464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M162"/>
+  <dimension ref="A1:M166"/>
   <sheetFormatPr defaultColWidth="25.44140625" defaultRowHeight="19.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.44140625" style="5"/>
@@ -2469,13 +2493,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
@@ -2495,13 +2519,13 @@
         <v>5</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
@@ -2528,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2536,7 +2560,7 @@
         <v>102</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>10</v>
@@ -2551,7 +2575,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2574,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2582,7 +2606,7 @@
         <v>104</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>12</v>
@@ -2597,7 +2621,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2614,13 +2638,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F7" s="5">
         <v>0</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2637,13 +2661,13 @@
         <v>1</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F8" s="5">
         <v>0</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2660,13 +2684,13 @@
         <v>2</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F9" s="5">
         <v>0</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2683,13 +2707,13 @@
         <v>3</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F10" s="5">
         <v>1</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2706,13 +2730,13 @@
         <v>3</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F11" s="5">
         <v>1</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2735,7 +2759,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2752,13 +2776,13 @@
         <v>2</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F13" s="5">
         <v>1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2781,7 +2805,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2804,7 +2828,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2827,7 +2851,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2850,7 +2874,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2867,13 +2891,13 @@
         <v>0</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F18" s="5">
         <v>0</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2890,13 +2914,13 @@
         <v>0</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="F19" s="5">
         <v>0</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2913,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="F20" s="5">
         <v>0</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2936,13 +2960,13 @@
         <v>0</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="F21" s="5">
         <v>0</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2959,13 +2983,13 @@
         <v>0</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="F22" s="5">
         <v>0</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2982,13 +3006,13 @@
         <v>1</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="F23" s="5">
         <v>0</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3005,13 +3029,13 @@
         <v>1</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F24" s="5">
         <v>0</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3028,13 +3052,13 @@
         <v>1</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="F25" s="5">
         <v>0</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3051,13 +3075,13 @@
         <v>1</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="F26" s="5">
         <v>0</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3074,13 +3098,13 @@
         <v>1</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F27" s="5">
         <v>0</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3097,13 +3121,13 @@
         <v>3</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="F28" s="5">
         <v>1</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3120,13 +3144,13 @@
         <v>2</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="F29" s="5">
         <v>0</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3143,13 +3167,13 @@
         <v>2</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F30" s="5">
         <v>0</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3166,13 +3190,13 @@
         <v>3</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F31" s="5">
         <v>1</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3195,7 +3219,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3218,7 +3242,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3241,7 +3265,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3264,7 +3288,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3287,7 +3311,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3310,7 +3334,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3333,7 +3357,7 @@
         <v>1</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3356,7 +3380,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3379,7 +3403,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3402,7 +3426,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3425,7 +3449,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3448,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3471,7 +3495,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3494,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3517,7 +3541,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3540,7 +3564,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3563,7 +3587,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3586,7 +3610,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3609,7 +3633,7 @@
         <v>1</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3632,7 +3656,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3655,7 +3679,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3678,7 +3702,7 @@
         <v>0</v>
       </c>
       <c r="G53" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3701,7 +3725,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3724,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3747,7 +3771,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3764,13 +3788,13 @@
         <v>1</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="F57" s="5">
         <v>0</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3793,7 +3817,7 @@
         <v>0</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3816,7 +3840,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3833,13 +3857,13 @@
         <v>1</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="F60" s="5">
         <v>1</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3862,7 +3886,7 @@
         <v>1</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3879,13 +3903,13 @@
         <v>2</v>
       </c>
       <c r="E62" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F62" s="5">
         <v>1</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3908,7 +3932,7 @@
         <v>0</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3931,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3954,7 +3978,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -3977,7 +4001,7 @@
         <v>0</v>
       </c>
       <c r="G66" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4000,7 +4024,7 @@
         <v>0</v>
       </c>
       <c r="G67" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4023,7 +4047,7 @@
         <v>1</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4046,7 +4070,7 @@
         <v>0</v>
       </c>
       <c r="G69" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4069,7 +4093,7 @@
         <v>0</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4092,7 +4116,7 @@
         <v>0</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4115,7 +4139,7 @@
         <v>0</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4138,7 +4162,7 @@
         <v>0</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4161,7 +4185,7 @@
         <v>0</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4184,7 +4208,7 @@
         <v>0</v>
       </c>
       <c r="G75" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4207,7 +4231,7 @@
         <v>0</v>
       </c>
       <c r="G76" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4230,7 +4254,7 @@
         <v>0</v>
       </c>
       <c r="G77" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4253,7 +4277,7 @@
         <v>0</v>
       </c>
       <c r="G78" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4276,7 +4300,7 @@
         <v>0</v>
       </c>
       <c r="G79" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4299,7 +4323,7 @@
         <v>0</v>
       </c>
       <c r="G80" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="81" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4322,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="G81" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4345,7 +4369,7 @@
         <v>0</v>
       </c>
       <c r="G82" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="83" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4368,7 +4392,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="84" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4391,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4414,7 +4438,7 @@
         <v>0</v>
       </c>
       <c r="G85" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4437,7 +4461,7 @@
         <v>0</v>
       </c>
       <c r="G86" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4460,7 +4484,7 @@
         <v>0</v>
       </c>
       <c r="G87" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4483,7 +4507,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4506,7 +4530,7 @@
         <v>0</v>
       </c>
       <c r="G89" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4529,7 +4553,7 @@
         <v>1</v>
       </c>
       <c r="G90" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4552,7 +4576,7 @@
         <v>0</v>
       </c>
       <c r="G91" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4575,7 +4599,7 @@
         <v>1</v>
       </c>
       <c r="G92" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4598,7 +4622,7 @@
         <v>1</v>
       </c>
       <c r="G93" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4621,7 +4645,7 @@
         <v>0</v>
       </c>
       <c r="G94" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4629,7 +4653,7 @@
         <v>193</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C95" s="5" t="s">
         <v>258</v>
@@ -4644,7 +4668,7 @@
         <v>0</v>
       </c>
       <c r="G95" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4667,7 +4691,7 @@
         <v>0</v>
       </c>
       <c r="G96" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4690,7 +4714,7 @@
         <v>0</v>
       </c>
       <c r="G97" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4713,7 +4737,7 @@
         <v>0</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4736,7 +4760,7 @@
         <v>1</v>
       </c>
       <c r="G99" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4759,7 +4783,7 @@
         <v>1</v>
       </c>
       <c r="G100" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4782,7 +4806,7 @@
         <v>0</v>
       </c>
       <c r="G101" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4805,7 +4829,7 @@
         <v>0</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4828,7 +4852,7 @@
         <v>0</v>
       </c>
       <c r="G103" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4851,7 +4875,7 @@
         <v>0</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4874,7 +4898,7 @@
         <v>1</v>
       </c>
       <c r="G105" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4897,7 +4921,7 @@
         <v>0</v>
       </c>
       <c r="G106" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4920,7 +4944,7 @@
         <v>0</v>
       </c>
       <c r="G107" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4943,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="G108" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4966,7 +4990,7 @@
         <v>0</v>
       </c>
       <c r="G109" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -4989,7 +5013,7 @@
         <v>0</v>
       </c>
       <c r="G110" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5012,7 +5036,7 @@
         <v>0</v>
       </c>
       <c r="G111" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5035,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="G112" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5058,7 +5082,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5081,7 +5105,7 @@
         <v>0</v>
       </c>
       <c r="G114" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5104,7 +5128,7 @@
         <v>0</v>
       </c>
       <c r="G115" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5127,7 +5151,7 @@
         <v>0</v>
       </c>
       <c r="G116" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5150,7 +5174,7 @@
         <v>1</v>
       </c>
       <c r="G117" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5173,7 +5197,7 @@
         <v>0</v>
       </c>
       <c r="G118" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5196,7 +5220,7 @@
         <v>0</v>
       </c>
       <c r="G119" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5219,7 +5243,7 @@
         <v>0</v>
       </c>
       <c r="G120" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5236,13 +5260,13 @@
         <v>3</v>
       </c>
       <c r="E121" s="5" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="F121" s="5">
         <v>0</v>
       </c>
       <c r="G121" s="5" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5265,7 +5289,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5288,7 +5312,7 @@
         <v>0</v>
       </c>
       <c r="G123" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5311,7 +5335,7 @@
         <v>0</v>
       </c>
       <c r="G124" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5334,7 +5358,7 @@
         <v>0</v>
       </c>
       <c r="G125" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5357,7 +5381,7 @@
         <v>0</v>
       </c>
       <c r="G126" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5368,19 +5392,19 @@
         <v>355</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D127" s="5">
         <v>1</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>356</v>
+        <v>496</v>
       </c>
       <c r="F127" s="5">
         <v>0</v>
       </c>
       <c r="G127" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5388,22 +5412,22 @@
         <v>226</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D128" s="5">
         <v>2</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F128" s="5">
         <v>1</v>
       </c>
       <c r="G128" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5411,22 +5435,22 @@
         <v>227</v>
       </c>
       <c r="B129" s="6" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D129" s="5">
         <v>1</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F129" s="5">
         <v>1</v>
       </c>
       <c r="G129" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5434,22 +5458,22 @@
         <v>228</v>
       </c>
       <c r="B130" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="C130" s="5" t="s">
         <v>364</v>
       </c>
-      <c r="C130" s="5" t="s">
-        <v>365</v>
-      </c>
       <c r="D130" s="5">
         <v>1</v>
       </c>
       <c r="E130" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F130" s="5">
         <v>0</v>
       </c>
       <c r="G130" s="5" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5457,22 +5481,22 @@
         <v>229</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D131" s="5">
         <v>2</v>
       </c>
       <c r="E131" s="5" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="F131" s="5">
         <v>0</v>
       </c>
       <c r="G131" s="5" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5480,22 +5504,22 @@
         <v>230</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D132" s="5">
         <v>1</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F132" s="5">
         <v>0</v>
       </c>
       <c r="G132" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5503,22 +5527,22 @@
         <v>231</v>
       </c>
       <c r="B133" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="D133" s="5">
+        <v>0</v>
+      </c>
+      <c r="E133" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="C133" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="D133" s="5">
-        <v>0</v>
-      </c>
-      <c r="E133" s="5" t="s">
-        <v>377</v>
-      </c>
       <c r="F133" s="5">
         <v>0</v>
       </c>
       <c r="G133" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5526,22 +5550,22 @@
         <v>232</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="D134" s="5">
         <v>0</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="F134" s="5">
         <v>0</v>
       </c>
       <c r="G134" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5549,22 +5573,22 @@
         <v>233</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D135" s="5">
         <v>0</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F135" s="5">
         <v>0</v>
       </c>
       <c r="G135" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5572,22 +5596,22 @@
         <v>234</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D136" s="5">
         <v>0</v>
       </c>
       <c r="E136" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F136" s="5">
         <v>0</v>
       </c>
       <c r="G136" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5595,22 +5619,22 @@
         <v>235</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D137" s="5">
         <v>0</v>
       </c>
       <c r="E137" s="5" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F137" s="5">
         <v>0</v>
       </c>
       <c r="G137" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5618,22 +5642,22 @@
         <v>236</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D138" s="5">
         <v>0</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F138" s="5">
         <v>0</v>
       </c>
       <c r="G138" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5641,22 +5665,22 @@
         <v>237</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D139" s="5">
         <v>0</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F139" s="5">
         <v>0</v>
       </c>
       <c r="G139" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5664,22 +5688,22 @@
         <v>238</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D140" s="5">
         <v>1</v>
       </c>
       <c r="E140" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F140" s="5">
         <v>0</v>
       </c>
       <c r="G140" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="141" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5687,22 +5711,22 @@
         <v>239</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D141" s="5">
         <v>1</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F141" s="5">
         <v>0</v>
       </c>
       <c r="G141" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5710,22 +5734,22 @@
         <v>240</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D142" s="5">
         <v>1</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F142" s="5">
         <v>0</v>
       </c>
       <c r="G142" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5733,22 +5757,22 @@
         <v>241</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D143" s="5">
         <v>1</v>
       </c>
       <c r="E143" s="5" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F143" s="5">
         <v>0</v>
       </c>
       <c r="G143" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="144" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5756,22 +5780,22 @@
         <v>242</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="D144" s="5">
         <v>1</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F144" s="5">
         <v>0</v>
       </c>
       <c r="G144" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="145" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5779,22 +5803,22 @@
         <v>243</v>
       </c>
       <c r="B145" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="D145" s="5">
+        <v>0</v>
+      </c>
+      <c r="E145" s="5" t="s">
         <v>413</v>
       </c>
-      <c r="C145" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="D145" s="5">
-        <v>0</v>
-      </c>
-      <c r="E145" s="5" t="s">
-        <v>414</v>
-      </c>
       <c r="F145" s="5">
         <v>0</v>
       </c>
       <c r="G145" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5802,22 +5826,22 @@
         <v>244</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D146" s="5">
         <v>0</v>
       </c>
       <c r="E146" s="5" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="F146" s="5">
         <v>0</v>
       </c>
       <c r="G146" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5825,22 +5849,22 @@
         <v>245</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D147" s="5">
         <v>0</v>
       </c>
       <c r="E147" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="F147" s="5">
         <v>0</v>
       </c>
       <c r="G147" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5848,22 +5872,22 @@
         <v>246</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D148" s="5">
         <v>1</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="F148" s="5">
         <v>0</v>
       </c>
       <c r="G148" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5871,22 +5895,22 @@
         <v>247</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="D149" s="5">
         <v>2</v>
       </c>
       <c r="E149" s="5" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F149" s="5">
         <v>1</v>
       </c>
       <c r="G149" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5894,22 +5918,22 @@
         <v>248</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="D150" s="5">
         <v>3</v>
       </c>
       <c r="E150" s="5" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F150" s="5">
         <v>1</v>
       </c>
       <c r="G150" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="151" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5917,22 +5941,22 @@
         <v>249</v>
       </c>
       <c r="B151" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="C151" s="5" t="s">
         <v>455</v>
       </c>
-      <c r="C151" s="5" t="s">
-        <v>456</v>
-      </c>
       <c r="D151" s="5">
         <v>1</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F151" s="5">
         <v>1</v>
       </c>
       <c r="G151" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5940,22 +5964,22 @@
         <v>250</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="D152" s="5">
         <v>1</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F152" s="5">
         <v>1</v>
       </c>
       <c r="G152" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="153" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5963,22 +5987,22 @@
         <v>251</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D153" s="5">
         <v>2</v>
       </c>
       <c r="E153" s="5" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F153" s="5">
         <v>1</v>
       </c>
       <c r="G153" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="154" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -5986,22 +6010,22 @@
         <v>252</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D154" s="5">
         <v>2</v>
       </c>
       <c r="E154" s="5" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F154" s="5">
         <v>0</v>
       </c>
       <c r="G154" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="155" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6009,22 +6033,22 @@
         <v>253</v>
       </c>
       <c r="B155" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="C155" s="5" t="s">
         <v>472</v>
-      </c>
-      <c r="C155" s="5" t="s">
-        <v>473</v>
       </c>
       <c r="D155" s="5">
         <v>3</v>
       </c>
       <c r="E155" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F155" s="5">
         <v>1</v>
       </c>
       <c r="G155" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="156" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6032,22 +6056,22 @@
         <v>254</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D156" s="5">
         <v>2</v>
       </c>
       <c r="E156" s="5" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F156" s="5">
         <v>1</v>
       </c>
       <c r="G156" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="157" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6055,22 +6079,22 @@
         <v>255</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D157" s="5">
         <v>3</v>
       </c>
       <c r="E157" s="5" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F157" s="5">
         <v>1</v>
       </c>
       <c r="G157" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="158" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6078,22 +6102,22 @@
         <v>256</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="D158" s="5">
         <v>3</v>
       </c>
       <c r="E158" s="5" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="F158" s="5">
         <v>1</v>
       </c>
       <c r="G158" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6101,22 +6125,22 @@
         <v>257</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C159" s="5" t="s">
+        <v>483</v>
+      </c>
+      <c r="D159" s="5">
+        <v>0</v>
+      </c>
+      <c r="E159" s="5" t="s">
         <v>484</v>
       </c>
-      <c r="D159" s="5">
-        <v>0</v>
-      </c>
-      <c r="E159" s="5" t="s">
-        <v>485</v>
-      </c>
       <c r="F159" s="5">
         <v>0</v>
       </c>
       <c r="G159" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6124,22 +6148,22 @@
         <v>258</v>
       </c>
       <c r="B160" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="C160" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="D160" s="5">
+        <v>1</v>
+      </c>
+      <c r="E160" s="5" t="s">
         <v>488</v>
       </c>
-      <c r="C160" s="5" t="s">
-        <v>487</v>
-      </c>
-      <c r="D160" s="5">
-        <v>1</v>
-      </c>
-      <c r="E160" s="5" t="s">
-        <v>489</v>
-      </c>
       <c r="F160" s="5">
         <v>0</v>
       </c>
       <c r="G160" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="161" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6147,22 +6171,22 @@
         <v>259</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="D161" s="5">
         <v>2</v>
       </c>
       <c r="E161" s="5" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="F161" s="5">
         <v>1</v>
       </c>
       <c r="G161" s="5" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="162" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -6170,23 +6194,75 @@
         <v>260</v>
       </c>
       <c r="B162" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="D162" s="5">
+        <v>1</v>
+      </c>
+      <c r="E162" s="5" t="s">
         <v>495</v>
       </c>
-      <c r="C162" s="5" t="s">
-        <v>496</v>
-      </c>
-      <c r="D162" s="5">
-        <v>1</v>
-      </c>
-      <c r="E162" s="5" t="s">
-        <v>497</v>
-      </c>
       <c r="F162" s="5">
         <v>1</v>
       </c>
       <c r="G162" s="5" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A163" s="5">
+        <v>261</v>
+      </c>
+      <c r="B163" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="C163" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="D163" s="5">
+        <v>2</v>
+      </c>
+      <c r="E163" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="F163" s="5">
+        <v>0</v>
+      </c>
+      <c r="G163" s="5" t="s">
         <v>441</v>
       </c>
+    </row>
+    <row r="164" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="5">
+        <v>262</v>
+      </c>
+      <c r="B164" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D164" s="5">
+        <v>0</v>
+      </c>
+      <c r="E164" s="5" t="s">
+        <v>502</v>
+      </c>
+      <c r="F164" s="5">
+        <v>1</v>
+      </c>
+      <c r="G164" s="5" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E165" s="5"/>
+    </row>
+    <row r="166" spans="1:7" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E166" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>